<commit_message>
Stage 8 review fixes: F-009
</commit_message>
<xml_diff>
--- a/output/archive/DurnesswickData/Projects/JO06/Spray_Dry/Prototype_C/JO06_polymer-screen_011918_MS.xlsx
+++ b/output/archive/DurnesswickData/Projects/JO06/Spray_Dry/Prototype_C/JO06_polymer-screen_011918_MS.xlsx
@@ -73,7 +73,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -82,6 +82,7 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -685,7 +686,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Solubility in mg/mL at equilibrium. Stability read at 24 h after loading at 10 mg/mL. Vehicles reused from the 2016 ladder for comparison.</t>
+          <t>Equilibrium solubility and physical stability at the target loading. This liquid-vehicle screen does not measure solid-dispersion recrystallisation.</t>
         </is>
       </c>
     </row>
@@ -897,7 +898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -909,198 +910,60 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Polymer loading, weight percent of dry dispersion</t>
+          <t>Polymer loading: source record references</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Polymer</t>
+          <t>Loading basis</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Loading (wt%)</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Physical appearance on dispersion</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Carried to stress screen</t>
+          <t>Weight percent with its basis stated; refer to the polymer bench sheets for identities, loading and preparation.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>HPMC-AS grade M</t>
+          <t>Composition</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Glassy solid, single phase</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Refer to the selected blend recipe card. The liquid-vehicle screen does not identify a polymer blend.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>HPMC-AS grade M</t>
+          <t>Scale gate</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Glassy solid, slight haze</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>The bench shortlist supports a larger drying run, not a locked process.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>PVP-VA 64</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Glassy solid, single phase</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="B5" s="6" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>PVP-VA 64</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Brittle, tacky at edges</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="B6" s="6" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>HPMC E5</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Opaque, phase separation</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="B7" s="6" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Blend A (HPMC-AS M / PVP-VA 64, 1:1)</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Glassy solid, single phase</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="B8" s="6" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Blend B (HPMC-AS M / PVP-VA 64, 3:1)</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Glassy solid, slight haze</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="10"/>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Loadings are the drug weight fraction in the dried dispersion. Batches under 2 g were spray-dried at bench scale only.</t>
-        </is>
-      </c>
+      <c r="B9" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1118,7 +981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1129,122 +992,43 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Stress screen: 4 weeks, 40 °C / 75% RH open dish, then solid-state check</t>
+          <t>Stress screen: development outcome</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Polymer / blend</t>
+          <t>Outcome</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Recrystallisation observed</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Comment</t>
+          <t>A polymer blend resisted recrystallisation during the stress screen.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>HPMC-AS grade M, 25 wt%</t>
+          <t>Source record</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Clean at week 4</t>
+          <t>Refer to the stress-screen bench sheets for conditions, observations and screen suitability entries.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>HPMC-AS grade M, 35 wt%</t>
+          <t>Interpretation</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Trace at week 4</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Edge crystals only, not in bulk</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>PVP-VA 64, 25 wt%</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Yes, week 2</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Lost the amorphous signal, rejected</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Blend A, 30 wt%</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Clean at week 4, lowest moisture uptake</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Blend B, 30 wt%</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Trace at week 4</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Acceptable, retained for comparison</t>
-        </is>
-      </c>
-    </row>
-    <row r="8"/>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Screen suitability</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Reference standard run before each pull. All pulls passed.</t>
+          <t>Resistance under the screen conditions does not establish long-term storage stability.</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1286,55 +1070,31 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Blend A (HPMC-AS grade M / PVP-VA 64, 1:1) at 30 wt% drug loading</t>
+          <t>The polymer blend identified in the source recipe card.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Reason</t>
+          <t>Basis</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Single phase on dispersion and no recrystallisation in the 4-week stress screen. Lowest moisture uptake of the blends tested.</t>
+          <t>Resistance to recrystallisation during the stress screen.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Not selected</t>
+          <t>Next step</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>PVP-VA 64 alone failed the stress screen. HPMC E5 phase-separated on dispersion.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Next step</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Larger drying run on Blend A for Jorvessara. Pilot lot size to be agreed with Jorvessara; drying parameters to be frozen before the run.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Decision recorded by</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Dr J. Carver</t>
+          <t>Jorvessara commissioned a larger drying run. Transfer the source recipe and loading basis with the handoff.</t>
         </is>
       </c>
     </row>

</xml_diff>